<commit_message>
Layout corrected: solenoid 44 is B3, not a second G3
The doubled G3 on solenoids 32 and 44 was a typo in the sheet; 44 is B3 (59).
The accompaniment rank is now nine pipes, C D E F G A Bb B C, and the
generator runs with no warnings.

One consequence worth recording: the all-notes sample file has always played a
B3 on Main, which the previous definition reported as a note the organ did not
have. It was never the file's error. The file's genuine errors are the four
that remain -- Main 28 and drums 23, 24 and 25.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/organ-arranger/instrument/layout.xlsx
+++ b/tools/organ-arranger/instrument/layout.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\massi\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BCF46AB-6753-4AB4-8451-0481F811450F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{239C8141-441D-4AC7-9572-AB783AAAC513}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1936,10 +1936,10 @@
         <v>44</v>
       </c>
       <c r="B46" s="18">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C46" s="32" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D46" s="19" t="s">
         <v>25</v>

</xml_diff>